<commit_message>
Save all absolute path and package fixes
</commit_message>
<xml_diff>
--- a/Diabetes_prediction_flask/user.xlsx
+++ b/Diabetes_prediction_flask/user.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -649,6 +649,74 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nithya</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nithyashreen124@gmail.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nithya@23</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Nithya</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nithyashreen125@gmail.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nithya@14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>navya</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>navyashreen037@gmail.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>navya@23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Nithya</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>navyashreen037@gmail.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Navya@21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>